<commit_message>
Fix D2 process-floor QFA and refresh downstream outputs
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_audit_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>key</t>
   </si>
@@ -31,6 +31,12 @@
     <t>mapping_version</t>
   </si>
   <si>
+    <t>qfa_window</t>
+  </si>
+  <si>
+    <t>process_floor_channels</t>
+  </si>
+  <si>
     <t>input_source</t>
   </si>
   <si>
@@ -64,25 +70,31 @@
     <t>input_time_base_contract.json_sha16</t>
   </si>
   <si>
-    <t>D2V1_20260710_1733</t>
-  </si>
-  <si>
-    <t>NorthBank_D2_v1_20260710</t>
-  </si>
-  <si>
-    <t>d2_v1_p0p1</t>
+    <t>D2V1_20260722_1714</t>
+  </si>
+  <si>
+    <t>NorthBank_D2_v1_20260722</t>
+  </si>
+  <si>
+    <t>d2_v1_process_floor_r1</t>
+  </si>
+  <si>
+    <t>6h</t>
+  </si>
+  <si>
+    <t>DO_1_4,DO_2_4</t>
   </si>
   <si>
     <t>1.1_time_base_contract</t>
   </si>
   <si>
-    <t>25d5e96846430518fe5f6400275f0b227b8f31bd5ca6ea57d4cddf8526c0c6ac</t>
-  </si>
-  <si>
-    <t>a28b5893bebbbe13</t>
-  </si>
-  <si>
-    <t>2026-07-10T17:34:27</t>
+    <t>130ae2acfa72e20acb455f8117f26b2ca95c9c51db98d1bf92b4802c4b74f6f7</t>
+  </si>
+  <si>
+    <t>ee468d139c4c71a0</t>
+  </si>
+  <si>
+    <t>2026-07-22T17:14:21</t>
   </si>
   <si>
     <t>f6296408c722c479</t>
@@ -443,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -459,7 +471,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -467,7 +479,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -475,7 +487,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -483,7 +495,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -491,7 +503,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -499,23 +511,23 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
-        <v>14</v>
+      <c r="B8" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9">
-        <v>6121</v>
+      <c r="B9" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -523,7 +535,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>45.88</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -531,7 +543,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>6121</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -539,31 +551,47 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>12.09</v>
+        <v>19.21</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" t="b">
-        <v>1</v>
+      <c r="B13">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
-        <v>22</v>
+      <c r="B14">
+        <v>6.4</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
-        <v>23</v>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize D2 scientific validation and hard availability semantics
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_audit_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>key</t>
   </si>
@@ -31,6 +31,21 @@
     <t>mapping_version</t>
   </si>
   <si>
+    <t>study_design_version</t>
+  </si>
+  <si>
+    <t>calibration_basis</t>
+  </si>
+  <si>
+    <t>temporal_integrity_source_scope</t>
+  </si>
+  <si>
+    <t>response_loss_role</t>
+  </si>
+  <si>
+    <t>external_site_validation</t>
+  </si>
+  <si>
     <t>qfa_window</t>
   </si>
   <si>
@@ -70,13 +85,28 @@
     <t>input_time_base_contract.json_sha16</t>
   </si>
   <si>
-    <t>D2V1_20260722_1714</t>
-  </si>
-  <si>
-    <t>NorthBank_D2_v1_20260722</t>
-  </si>
-  <si>
-    <t>d2_v1_process_floor_r1</t>
+    <t>D2V2_20260804_1823</t>
+  </si>
+  <si>
+    <t>NorthBank_D2_v2_20260804</t>
+  </si>
+  <si>
+    <t>d2_v2_hard_availability_r1</t>
+  </si>
+  <si>
+    <t>d2_blocked_time_v1</t>
+  </si>
+  <si>
+    <t>blocked_development_reference_v2</t>
+  </si>
+  <si>
+    <t>source_file_global_plus_channel_missingness</t>
+  </si>
+  <si>
+    <t>diagnostic_only</t>
+  </si>
+  <si>
+    <t>deferred</t>
   </si>
   <si>
     <t>6h</t>
@@ -88,13 +118,13 @@
     <t>1.1_time_base_contract</t>
   </si>
   <si>
-    <t>130ae2acfa72e20acb455f8117f26b2ca95c9c51db98d1bf92b4802c4b74f6f7</t>
-  </si>
-  <si>
-    <t>ee468d139c4c71a0</t>
-  </si>
-  <si>
-    <t>2026-07-22T17:14:21</t>
+    <t>7ea42ecbec15d8a715422f8d7356c163572a647aa4aecb573932aaa4bcb3ccdd</t>
+  </si>
+  <si>
+    <t>4dbc7a25415d4d5d</t>
+  </si>
+  <si>
+    <t>2026-08-04T18:23:22</t>
   </si>
   <si>
     <t>f6296408c722c479</t>
@@ -455,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -471,7 +501,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -479,7 +509,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -487,7 +517,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -495,7 +525,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -503,7 +533,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -511,7 +541,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -519,7 +549,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -527,71 +557,111 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10">
-        <v>14</v>
+      <c r="B10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11">
-        <v>6121</v>
+      <c r="B11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12">
-        <v>19.21</v>
+      <c r="B12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13">
-        <v>0</v>
+      <c r="B13" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14">
-        <v>6.4</v>
+      <c r="B14" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" t="b">
-        <v>1</v>
+      <c r="B15">
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" t="s">
-        <v>26</v>
+      <c r="B16">
+        <v>6121</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
-      <c r="B17" t="s">
-        <v>27</v>
+      <c r="B17">
+        <v>10.72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>3649</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct D2 raw timestamp integrity scoring
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_audit_log.xlsx
@@ -85,19 +85,19 @@
     <t>input_time_base_contract.json_sha16</t>
   </si>
   <si>
-    <t>D2V2_20260804_1823</t>
-  </si>
-  <si>
-    <t>NorthBank_D2_v2_20260804</t>
-  </si>
-  <si>
-    <t>d2_v2_hard_availability_r1</t>
+    <t>D2V3_20260804_1939</t>
+  </si>
+  <si>
+    <t>NorthBank_D2_v3_20260804</t>
+  </si>
+  <si>
+    <t>d2_v3_source_timestamp_qti_r1</t>
   </si>
   <si>
     <t>d2_blocked_time_v1</t>
   </si>
   <si>
-    <t>blocked_development_reference_v2</t>
+    <t>blocked_development_reference_v3</t>
   </si>
   <si>
     <t>source_file_global_plus_channel_missingness</t>
@@ -118,13 +118,13 @@
     <t>1.1_time_base_contract</t>
   </si>
   <si>
-    <t>7ea42ecbec15d8a715422f8d7356c163572a647aa4aecb573932aaa4bcb3ccdd</t>
-  </si>
-  <si>
-    <t>4dbc7a25415d4d5d</t>
-  </si>
-  <si>
-    <t>2026-08-04T18:23:22</t>
+    <t>c492b1f1079e81d4de557fcea966741f4a8f4fe39769e2d1504718f11896a8db</t>
+  </si>
+  <si>
+    <t>3e3868b4c96a90c4</t>
+  </si>
+  <si>
+    <t>2026-08-04T19:40:17</t>
   </si>
   <si>
     <t>f6296408c722c479</t>
@@ -621,7 +621,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>10.72</v>
+        <v>52.79</v>
       </c>
     </row>
     <row r="18" spans="1:2">

</xml_diff>